<commit_message>
Upload GitHub Summary - 2026-09-15 01:32:10
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 14, 2026</t>
+    <t>September 15, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3229</v>
+        <v>3233</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>184</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-09-17 01:30:37
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 16, 2026</t>
+    <t>September 17, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3233</v>
+        <v>3234</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-09-22 01:29:50
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 21, 2026</t>
+    <t>September 22, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3234</v>
+        <v>3238</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-09-23 01:29:32
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 22, 2026</t>
+    <t>September 23, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3238</v>
+        <v>3240</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-09-24 01:30:17
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 23, 2026</t>
+    <t>September 24, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3240</v>
+        <v>3242</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-09-25 01:29:40
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 24, 2026</t>
+    <t>September 25, 2026</t>
   </si>
 </sst>
 </file>
@@ -497,7 +497,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -515,7 +515,7 @@
         <v>46</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3242</v>
+        <v>3244</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-09-26 01:28:25
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 25, 2026</t>
+    <t>September 26, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3244</v>
+        <v>3245</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-09-29 01:34:56
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 28, 2026</t>
+    <t>September 29, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3245</v>
+        <v>3248</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-09-30 01:37:26
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 29, 2026</t>
+    <t>September 30, 2026</t>
   </si>
 </sst>
 </file>
@@ -627,7 +627,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -645,7 +645,7 @@
         <v>13</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3248</v>
+        <v>3250</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -886,7 +886,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -904,7 +904,7 @@
         <v>23</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-10-01 01:44:36
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>September 30, 2026</t>
+    <t>October 1, 2026</t>
   </si>
 </sst>
 </file>
@@ -601,7 +601,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C6">
         <v>8</v>
@@ -619,7 +619,7 @@
         <v>1</v>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -860,7 +860,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C6">
         <v>40</v>
@@ -878,7 +878,7 @@
         <v>1</v>
       </c>
       <c r="H6">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-10-02 01:36:29
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 1, 2026</t>
+    <t>October 2, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3250</v>
+        <v>3251</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-10-07 01:39:40
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 6, 2026</t>
+    <t>October 7, 2026</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3251</v>
+        <v>3253</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" spans="1:8">

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-10-09 01:41:31
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 8, 2026</t>
+    <t>October 9, 2026</t>
   </si>
 </sst>
 </file>
@@ -689,7 +689,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -707,7 +707,7 @@
         <v>12</v>
       </c>
       <c r="H11">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3253</v>
+        <v>3255</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -948,7 +948,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -966,7 +966,7 @@
         <v>48</v>
       </c>
       <c r="H11">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload GitHub Summary - 2026-10-19 11:44:35
</commit_message>
<xml_diff>
--- a/assets/gitmetrics_growth_summary.xlsx
+++ b/assets/gitmetrics_growth_summary.xlsx
@@ -100,7 +100,7 @@
     <t>date</t>
   </si>
   <si>
-    <t>October 9, 2026</t>
+    <t>October 19, 2026</t>
   </si>
 </sst>
 </file>
@@ -497,7 +497,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="C2">
         <v>130</v>
@@ -515,7 +515,7 @@
         <v>46</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -658,7 +658,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C9">
         <v>20</v>
@@ -676,7 +676,7 @@
         <v>4</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -756,7 +756,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>3255</v>
+        <v>3261</v>
       </c>
       <c r="C2">
         <v>486</v>
@@ -774,7 +774,7 @@
         <v>376</v>
       </c>
       <c r="H2">
-        <v>210</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -917,7 +917,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C9">
         <v>54</v>
@@ -935,7 +935,7 @@
         <v>4</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -948,7 +948,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -966,7 +966,7 @@
         <v>48</v>
       </c>
       <c r="H11">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -1060,7 +1060,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>